<commit_message>
Group placeholder store categories as Uncategorized
The store files 219 products under placeholder category names
("Default", "Add a comment"). The report now groups them as
"Uncategorized" so category stats reflect real categories. Raw
crawl output is unchanged. Also refreshes all sample outputs from
a new run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-login-infinite-scroll-playwright/output/quotes.xlsx
+++ b/02-login-infinite-scroll-playwright/output/quotes.xlsx
@@ -765,147 +765,147 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>I love you without knowing how, or when, or from where. I love you simply, without problems or pride: I love you in this way because I do not know any other way of loving but this, in which there is no I or you, so intimate that your hand upon my chest is my hand, so intimate that when I fall asleep your eyes close.</t>
+          <t>This life is what you make it. No matter what, you're going to mess up sometimes, it's a universal truth. But the good part is you get to decide how you're going to mess it up. Girls will be your friends - they'll act like it anyway. But just remember, some come, some go. The ones that stay with you through everything - they're your true best friends. Don't let go of them. Also remember, sisters make the best friends in the world. As for lovers, well, they'll come and go too. And baby, I hate to say it, most of them - actually pretty much all of them are going to break your heart, but you can't give up because if you give up, you'll never find your soulmate. You'll never find that half who makes you whole and that goes for everything. Just because you fail once, doesn't mean you're gonna fail at everything. Keep trying, hold on, and always, always, always believe in yourself, because if you don't, then who will, sweetie? So keep your head high, keep your chin up, and most importantly, keep smiling, because life's a beautiful thing and there's so much to smile about.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pablo Neruda</t>
+          <t>Marilyn Monroe</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>love, poetry</t>
+          <t>friends, heartbreak, inspirational, life, love, sisters</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/4026.Pablo_Neruda</t>
+          <t>http://goodreads.com/author/show/82952.Marilyn_Monroe</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Pablo-Neruda</t>
+          <t>https://quotes.toscrape.com/author/Marilyn-Monroe</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>For every minute you are angry you lose sixty seconds of happiness.</t>
+          <t>It takes a great deal of bravery to stand up to our enemies, but just as much to stand up to our friends.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ralph Waldo Emerson</t>
+          <t>J.K. Rowling</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>happiness</t>
+          <t>courage, friends</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/12080.Ralph_Waldo_Emerson</t>
+          <t>http://goodreads.com/author/show/1077326.J_K_Rowling</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Ralph-Waldo-Emerson</t>
+          <t>https://quotes.toscrape.com/author/J-K-Rowling</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>If you judge people, you have no time to love them.</t>
+          <t>If you can't explain it to a six year old, you don't understand it yourself.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mother Teresa</t>
+          <t>Albert Einstein</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>attributed-no-source</t>
+          <t>simplicity, understand</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/838305.Mother_Teresa</t>
+          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Mother-Teresa</t>
+          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Anyone who thinks sitting in church can make you a Christian must also think that sitting in a garage can make you a car.</t>
+          <t>You may not be her first, her last, or her only. She loved before she may love again. But if she loves you now, what else matters? She's not perfect—you aren't either, and the two of you may never be perfect together but if she can make you laugh, cause you to think twice, and admit to being human and making mistakes, hold onto her and give her the most you can. She may not be thinking about you every second of the day, but she will give you a part of her that she knows you can break—her heart. So don't hurt her, don't change her, don't analyze and don't expect more than she can give. Smile when she makes you happy, let her know when she makes you mad, and miss her when she's not there.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Garrison Keillor</t>
+          <t>Bob Marley</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>humor, religion</t>
+          <t>love</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/2014.Garrison_Keillor</t>
+          <t>http://goodreads.com/author/show/25241.Bob_Marley</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Garrison-Keillor</t>
+          <t>https://quotes.toscrape.com/author/Bob-Marley</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Beauty is in the eye of the beholder and it may be necessary from time to time to give a stupid or misinformed beholder a black eye.</t>
+          <t>I like nonsense, it wakes up the brain cells. Fantasy is a necessary ingredient in living.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jim Henson</t>
+          <t>Dr. Seuss</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>humor</t>
+          <t>fantasy</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/4427.Jim_Henson</t>
+          <t>http://goodreads.com/author/show/61105.Dr_Seuss</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Jim-Henson</t>
+          <t>https://quotes.toscrape.com/author/Dr-Seuss</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -915,203 +915,207 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Today you are You, that is truer than true. There is no one alive who is Youer than You.</t>
+          <t>I may not have gone where I intended to go, but I think I have ended up where I needed to be.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dr. Seuss</t>
+          <t>Douglas Adams</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>comedy, life, yourself</t>
+          <t>life, navigation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/61105.Dr_Seuss</t>
+          <t>http://goodreads.com/author/show/4.Douglas_Adams</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Dr-Seuss</t>
+          <t>https://quotes.toscrape.com/author/Douglas-Adams</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>If you want your children to be intelligent, read them fairy tales. If you want them to be more intelligent, read them more fairy tales.</t>
+          <t>The opposite of love is not hate, it's indifference. The opposite of art is not ugliness, it's indifference. The opposite of faith is not heresy, it's indifference. And the opposite of life is not death, it's indifference.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Albert Einstein</t>
+          <t>Elie Wiesel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>children, fairy-tales</t>
+          <t>activism, apathy, hate, indifference, inspirational, love, opposite, philosophy</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
+          <t>http://goodreads.com/author/show/1049.Elie_Wiesel</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
+          <t>https://quotes.toscrape.com/author/Elie-Wiesel</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>It is impossible to live without failing at something, unless you live so cautiously that you might as well not have lived at all - in which case, you fail by default.</t>
+          <t>It is not a lack of love, but a lack of friendship that makes unhappy marriages.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>J.K. Rowling</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>Friedrich Nietzsche</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>friendship, lack-of-friendship, lack-of-love, love, marriage, unhappy-marriage</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/1077326.J_K_Rowling</t>
+          <t>http://goodreads.com/author/show/1938.Friedrich_Nietzsche</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/J-K-Rowling</t>
+          <t>https://quotes.toscrape.com/author/Friedrich-Nietzsche</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Logic will get you from A to Z; imagination will get you everywhere.</t>
+          <t>Good friends, good books, and a sleepy conscience: this is the ideal life.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Albert Einstein</t>
+          <t>Mark Twain</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>imagination</t>
+          <t>books, contentment, friends, friendship, life</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
+          <t>http://goodreads.com/author/show/1244.Mark_Twain</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
+          <t>https://quotes.toscrape.com/author/Mark-Twain</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>One good thing about music, when it hits you, you feel no pain.</t>
+          <t>Life is what happens to us while we are making other plans.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bob Marley</t>
+          <t>Allen Saunders</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>music</t>
+          <t>fate, life, misattributed-john-lennon, planning, plans</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/25241.Bob_Marley</t>
+          <t>http://goodreads.com/author/show/276029.Allen_Saunders</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Bob-Marley</t>
+          <t>https://quotes.toscrape.com/author/Allen-Saunders</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>The more that you read, the more things you will know. The more that you learn, the more places you'll go.</t>
+          <t>I love you without knowing how, or when, or from where. I love you simply, without problems or pride: I love you in this way because I do not know any other way of loving but this, in which there is no I or you, so intimate that your hand upon my chest is my hand, so intimate that when I fall asleep your eyes close.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dr. Seuss</t>
+          <t>Pablo Neruda</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>learning, reading, seuss</t>
+          <t>love, poetry</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/61105.Dr_Seuss</t>
+          <t>http://goodreads.com/author/show/4026.Pablo_Neruda</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Dr-Seuss</t>
+          <t>https://quotes.toscrape.com/author/Pablo-Neruda</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Of course it is happening inside your head, Harry, but why on earth should that mean that it is not real?</t>
+          <t>For every minute you are angry you lose sixty seconds of happiness.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>J.K. Rowling</t>
+          <t>Ralph Waldo Emerson</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>dumbledore</t>
+          <t>happiness</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/1077326.J_K_Rowling</t>
+          <t>http://goodreads.com/author/show/12080.Ralph_Waldo_Emerson</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/J-K-Rowling</t>
+          <t>https://quotes.toscrape.com/author/Ralph-Waldo-Emerson</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1121,27 +1125,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>The truth is, everyone is going to hurt you. You just got to find the ones worth suffering for.</t>
+          <t>If you judge people, you have no time to love them.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bob Marley</t>
+          <t>Mother Teresa</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>friendship</t>
+          <t>attributed-no-source</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/25241.Bob_Marley</t>
+          <t>http://goodreads.com/author/show/838305.Mother_Teresa</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Bob-Marley</t>
+          <t>https://quotes.toscrape.com/author/Mother-Teresa</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1151,27 +1155,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Not all of us can do great things. But we can do small things with great love.</t>
+          <t>Anyone who thinks sitting in church can make you a Christian must also think that sitting in a garage can make you a car.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mother Teresa</t>
+          <t>Garrison Keillor</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>misattributed-to-mother-teresa, paraphrased</t>
+          <t>humor, religion</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/838305.Mother_Teresa</t>
+          <t>http://goodreads.com/author/show/2014.Garrison_Keillor</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Mother-Teresa</t>
+          <t>https://quotes.toscrape.com/author/Garrison-Keillor</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1181,57 +1185,57 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>To the well-organized mind, death is but the next great adventure.</t>
+          <t>Beauty is in the eye of the beholder and it may be necessary from time to time to give a stupid or misinformed beholder a black eye.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>J.K. Rowling</t>
+          <t>Jim Henson</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>death, inspirational</t>
+          <t>humor</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/1077326.J_K_Rowling</t>
+          <t>http://goodreads.com/author/show/4427.Jim_Henson</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/J-K-Rowling</t>
+          <t>https://quotes.toscrape.com/author/Jim-Henson</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>All you need is love. But a little chocolate now and then doesn't hurt.</t>
+          <t>Today you are You, that is truer than true. There is no one alive who is Youer than You.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Charles M. Schulz</t>
+          <t>Dr. Seuss</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>chocolate, food, humor</t>
+          <t>comedy, life, yourself</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/209672.Charles_M_Schulz</t>
+          <t>http://goodreads.com/author/show/61105.Dr_Seuss</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Charles-M-Schulz</t>
+          <t>https://quotes.toscrape.com/author/Dr-Seuss</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1241,27 +1245,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>We read to know we're not alone.</t>
+          <t>If you want your children to be intelligent, read them fairy tales. If you want them to be more intelligent, read them more fairy tales.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>William Nicholson</t>
+          <t>Albert Einstein</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>misattributed-to-c-s-lewis, reading</t>
+          <t>children, fairy-tales</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/46130.William_Nicholson</t>
+          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/William-Nicholson</t>
+          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1271,87 +1275,83 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Any fool can know. The point is to understand.</t>
+          <t>It is impossible to live without failing at something, unless you live so cautiously that you might as well not have lived at all - in which case, you fail by default.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Albert Einstein</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>knowledge, learning, understanding, wisdom</t>
-        </is>
-      </c>
+          <t>J.K. Rowling</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
+          <t>http://goodreads.com/author/show/1077326.J_K_Rowling</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
+          <t>https://quotes.toscrape.com/author/J-K-Rowling</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>I have always imagined that Paradise will be a kind of library.</t>
+          <t>Logic will get you from A to Z; imagination will get you everywhere.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jorge Luis Borges</t>
+          <t>Albert Einstein</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>books, library</t>
+          <t>imagination</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/500.Jorge_Luis_Borges</t>
+          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Jorge-Luis-Borges</t>
+          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>It is never too late to be what you might have been.</t>
+          <t>One good thing about music, when it hits you, you feel no pain.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>George Eliot</t>
+          <t>Bob Marley</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>inspirational</t>
+          <t>music</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/173.George_Eliot</t>
+          <t>http://goodreads.com/author/show/25241.Bob_Marley</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/George-Eliot</t>
+          <t>https://quotes.toscrape.com/author/Bob-Marley</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1361,37 +1361,37 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>This life is what you make it. No matter what, you're going to mess up sometimes, it's a universal truth. But the good part is you get to decide how you're going to mess it up. Girls will be your friends - they'll act like it anyway. But just remember, some come, some go. The ones that stay with you through everything - they're your true best friends. Don't let go of them. Also remember, sisters make the best friends in the world. As for lovers, well, they'll come and go too. And baby, I hate to say it, most of them - actually pretty much all of them are going to break your heart, but you can't give up because if you give up, you'll never find your soulmate. You'll never find that half who makes you whole and that goes for everything. Just because you fail once, doesn't mean you're gonna fail at everything. Keep trying, hold on, and always, always, always believe in yourself, because if you don't, then who will, sweetie? So keep your head high, keep your chin up, and most importantly, keep smiling, because life's a beautiful thing and there's so much to smile about.</t>
+          <t>The more that you read, the more things you will know. The more that you learn, the more places you'll go.</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Marilyn Monroe</t>
+          <t>Dr. Seuss</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>friends, heartbreak, inspirational, life, love, sisters</t>
+          <t>learning, reading, seuss</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/82952.Marilyn_Monroe</t>
+          <t>http://goodreads.com/author/show/61105.Dr_Seuss</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Marilyn-Monroe</t>
+          <t>https://quotes.toscrape.com/author/Dr-Seuss</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>It takes a great deal of bravery to stand up to our enemies, but just as much to stand up to our friends.</t>
+          <t>Of course it is happening inside your head, Harry, but why on earth should that mean that it is not real?</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>courage, friends</t>
+          <t>dumbledore</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1415,247 +1415,247 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>If you can't explain it to a six year old, you don't understand it yourself.</t>
+          <t>The truth is, everyone is going to hurt you. You just got to find the ones worth suffering for.</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Albert Einstein</t>
+          <t>Bob Marley</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>simplicity, understand</t>
+          <t>friendship</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
+          <t>http://goodreads.com/author/show/25241.Bob_Marley</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
+          <t>https://quotes.toscrape.com/author/Bob-Marley</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>You may not be her first, her last, or her only. She loved before she may love again. But if she loves you now, what else matters? She's not perfect—you aren't either, and the two of you may never be perfect together but if she can make you laugh, cause you to think twice, and admit to being human and making mistakes, hold onto her and give her the most you can. She may not be thinking about you every second of the day, but she will give you a part of her that she knows you can break—her heart. So don't hurt her, don't change her, don't analyze and don't expect more than she can give. Smile when she makes you happy, let her know when she makes you mad, and miss her when she's not there.</t>
+          <t>Not all of us can do great things. But we can do small things with great love.</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Bob Marley</t>
+          <t>Mother Teresa</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>love</t>
+          <t>misattributed-to-mother-teresa, paraphrased</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/25241.Bob_Marley</t>
+          <t>http://goodreads.com/author/show/838305.Mother_Teresa</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Bob-Marley</t>
+          <t>https://quotes.toscrape.com/author/Mother-Teresa</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>I like nonsense, it wakes up the brain cells. Fantasy is a necessary ingredient in living.</t>
+          <t>To the well-organized mind, death is but the next great adventure.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dr. Seuss</t>
+          <t>J.K. Rowling</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>fantasy</t>
+          <t>death, inspirational</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/61105.Dr_Seuss</t>
+          <t>http://goodreads.com/author/show/1077326.J_K_Rowling</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Dr-Seuss</t>
+          <t>https://quotes.toscrape.com/author/J-K-Rowling</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>I may not have gone where I intended to go, but I think I have ended up where I needed to be.</t>
+          <t>All you need is love. But a little chocolate now and then doesn't hurt.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Douglas Adams</t>
+          <t>Charles M. Schulz</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>life, navigation</t>
+          <t>chocolate, food, humor</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/4.Douglas_Adams</t>
+          <t>http://goodreads.com/author/show/209672.Charles_M_Schulz</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Douglas-Adams</t>
+          <t>https://quotes.toscrape.com/author/Charles-M-Schulz</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>The opposite of love is not hate, it's indifference. The opposite of art is not ugliness, it's indifference. The opposite of faith is not heresy, it's indifference. And the opposite of life is not death, it's indifference.</t>
+          <t>We read to know we're not alone.</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Elie Wiesel</t>
+          <t>William Nicholson</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>activism, apathy, hate, indifference, inspirational, love, opposite, philosophy</t>
+          <t>misattributed-to-c-s-lewis, reading</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/1049.Elie_Wiesel</t>
+          <t>http://goodreads.com/author/show/46130.William_Nicholson</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Elie-Wiesel</t>
+          <t>https://quotes.toscrape.com/author/William-Nicholson</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>It is not a lack of love, but a lack of friendship that makes unhappy marriages.</t>
+          <t>Any fool can know. The point is to understand.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Friedrich Nietzsche</t>
+          <t>Albert Einstein</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>friendship, lack-of-friendship, lack-of-love, love, marriage, unhappy-marriage</t>
+          <t>knowledge, learning, understanding, wisdom</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/1938.Friedrich_Nietzsche</t>
+          <t>http://goodreads.com/author/show/9810.Albert_Einstein</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Friedrich-Nietzsche</t>
+          <t>https://quotes.toscrape.com/author/Albert-Einstein</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Good friends, good books, and a sleepy conscience: this is the ideal life.</t>
+          <t>I have always imagined that Paradise will be a kind of library.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Mark Twain</t>
+          <t>Jorge Luis Borges</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>books, contentment, friends, friendship, life</t>
+          <t>books, library</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/1244.Mark_Twain</t>
+          <t>http://goodreads.com/author/show/500.Jorge_Luis_Borges</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Mark-Twain</t>
+          <t>https://quotes.toscrape.com/author/Jorge-Luis-Borges</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Life is what happens to us while we are making other plans.</t>
+          <t>It is never too late to be what you might have been.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Allen Saunders</t>
+          <t>George Eliot</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>fate, life, misattributed-john-lennon, planning, plans</t>
+          <t>inspirational</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>http://goodreads.com/author/show/276029.Allen_Saunders</t>
+          <t>http://goodreads.com/author/show/173.George_Eliot</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://quotes.toscrape.com/author/Allen-Saunders</t>
+          <t>https://quotes.toscrape.com/author/George-Eliot</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -4431,7 +4431,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>religion</t>
+          <t>courage</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4441,7 +4441,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>yourself</t>
+          <t>philosophy</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -4451,7 +4451,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>children</t>
+          <t>religion</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -4461,7 +4461,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>music</t>
+          <t>yourself</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -4471,7 +4471,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>children</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -4481,7 +4481,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>dumbledore</t>
+          <t>music</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -4491,7 +4491,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>library</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -4501,7 +4501,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>courage</t>
+          <t>dumbledore</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -4511,7 +4511,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>philosophy</t>
+          <t>library</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -4701,7 +4701,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>poetry</t>
+          <t>heartbreak</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -4711,7 +4711,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>happiness</t>
+          <t>sisters</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -4721,7 +4721,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>comedy</t>
+          <t>simplicity</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -4731,7 +4731,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fairy-tales</t>
+          <t>understand</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -4741,7 +4741,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>imagination</t>
+          <t>fantasy</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -4751,7 +4751,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>seuss</t>
+          <t>navigation</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -4761,7 +4761,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>misattributed-to-mother-teresa</t>
+          <t>activism</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -4771,7 +4771,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>chocolate</t>
+          <t>apathy</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -4781,7 +4781,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>food</t>
+          <t>hate</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -4791,7 +4791,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>misattributed-to-c-s-lewis</t>
+          <t>indifference</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -4801,7 +4801,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>knowledge</t>
+          <t>opposite</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4811,7 +4811,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>understanding</t>
+          <t>lack-of-friendship</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4821,7 +4821,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>wisdom</t>
+          <t>lack-of-love</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4831,7 +4831,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>heartbreak</t>
+          <t>marriage</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4841,7 +4841,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>sisters</t>
+          <t>unhappy-marriage</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4851,7 +4851,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>simplicity</t>
+          <t>contentment</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4861,7 +4861,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>understand</t>
+          <t>fate</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4871,7 +4871,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>fantasy</t>
+          <t>misattributed-john-lennon</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4881,7 +4881,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>planning</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4891,7 +4891,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>activism</t>
+          <t>plans</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4901,7 +4901,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>apathy</t>
+          <t>poetry</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -4911,7 +4911,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>hate</t>
+          <t>happiness</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -4921,7 +4921,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>indifference</t>
+          <t>comedy</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -4931,7 +4931,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>opposite</t>
+          <t>fairy-tales</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -4941,7 +4941,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>lack-of-friendship</t>
+          <t>imagination</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -4951,7 +4951,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>lack-of-love</t>
+          <t>seuss</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -4961,7 +4961,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>marriage</t>
+          <t>misattributed-to-mother-teresa</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -4971,7 +4971,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>unhappy-marriage</t>
+          <t>chocolate</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -4981,7 +4981,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>contentment</t>
+          <t>food</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -4991,7 +4991,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>fate</t>
+          <t>misattributed-to-c-s-lewis</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -5001,7 +5001,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>misattributed-john-lennon</t>
+          <t>knowledge</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -5011,7 +5011,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>planning</t>
+          <t>understanding</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -5021,7 +5021,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>plans</t>
+          <t>wisdom</t>
         </is>
       </c>
       <c r="B77" t="n">

</xml_diff>